<commit_message>
Phase 1 complete: Quote-based system backend + customer UI - Migration script, quote controller, API routes, customer pages
</commit_message>
<xml_diff>
--- a/backend/data/order_items.xlsx
+++ b/backend/data/order_items.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:P5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -425,7 +425,28 @@
         <v>created_at</v>
       </c>
       <c r="I1" t="str">
-        <v>medicine_id</v>
+        <v>admin_set_price</v>
+      </c>
+      <c r="J1" t="str">
+        <v>original_price</v>
+      </c>
+      <c r="K1" t="str">
+        <v>discount_percent</v>
+      </c>
+      <c r="L1" t="str">
+        <v>customer_notes</v>
+      </c>
+      <c r="M1" t="str">
+        <v>admin_notes</v>
+      </c>
+      <c r="N1" t="str">
+        <v>is_substitution</v>
+      </c>
+      <c r="O1" t="str">
+        <v>price_locked</v>
+      </c>
+      <c r="P1" t="str">
+        <v>substitution_for</v>
       </c>
     </row>
     <row r="2">
@@ -453,6 +474,27 @@
       <c r="H2" t="str">
         <v>2026-03-13T09:46:39.331Z</v>
       </c>
+      <c r="I2">
+        <v>25</v>
+      </c>
+      <c r="J2">
+        <v>25</v>
+      </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2" t="b">
+        <v>0</v>
+      </c>
+      <c r="O2" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -479,6 +521,27 @@
       <c r="H3" t="str">
         <v>2026-03-13T09:46:46.626Z</v>
       </c>
+      <c r="I3">
+        <v>25</v>
+      </c>
+      <c r="J3">
+        <v>25</v>
+      </c>
+      <c r="K3">
+        <v>0</v>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="b">
+        <v>0</v>
+      </c>
+      <c r="O3" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -505,6 +568,27 @@
       <c r="H4" t="str">
         <v>2026-03-13T09:54:18.615Z</v>
       </c>
+      <c r="I4">
+        <v>25</v>
+      </c>
+      <c r="J4">
+        <v>25</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v/>
+      </c>
+      <c r="N4" t="b">
+        <v>0</v>
+      </c>
+      <c r="O4" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -531,10 +615,31 @@
       <c r="H5" t="str">
         <v>2026-03-13T09:54:32.578Z</v>
       </c>
+      <c r="I5">
+        <v>25</v>
+      </c>
+      <c r="J5">
+        <v>25</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v/>
+      </c>
+      <c r="N5" t="b">
+        <v>0</v>
+      </c>
+      <c r="O5" t="b">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>